<commit_message>
change object student,user and add code insert list student(have config scheulde send mail and insert account) and add file excel template sample for insert list student
</commit_message>
<xml_diff>
--- a/src/main/resources/static/example_insert_list_student.xlsx
+++ b/src/main/resources/static/example_insert_list_student.xlsx
@@ -1,21 +1,20 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr6="http://schemas.microsoft.com/office/spreadsheetml/2016/revision6" xmlns:xr10="http://schemas.microsoft.com/office/spreadsheetml/2016/revision10" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" mc:Ignorable="x15 xr xr6 xr10 xr2">
-  <fileVersion appName="xl" lastEdited="7" lowestEdited="7" rupBuild="29127"/>
-  <workbookPr defaultThemeVersion="166925"/>
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" mc:Ignorable="x15">
+  <fileVersion appName="xl" lastEdited="6" lowestEdited="6" rupBuild="14420"/>
+  <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="D:\study\document\do_an_tot_nghiep\do_an\document\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PC\Documents\do_an\back-end\DATN\src\main\resources\static\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B01B9842-1C76-4102-8AEC-C2B5CB676029}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="4815" yWindow="2250" windowWidth="22170" windowHeight="11340" xr2:uid="{C798A28C-3069-4D61-822A-CAD72978DBE0}"/>
+    <workbookView xWindow="4815" yWindow="2250" windowWidth="22170" windowHeight="11340"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
-  <calcPr calcId="191028"/>
+  <calcPr calcId="152511"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -25,7 +24,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="10" uniqueCount="10">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="11" uniqueCount="11">
   <si>
     <t>No.</t>
   </si>
@@ -87,30 +86,19 @@
     <t>CCCD/CMND</t>
   </si>
   <si>
-    <r>
-      <t xml:space="preserve">Chuyên nghành </t>
-    </r>
-    <r>
-      <rPr>
-        <b/>
-        <sz val="11"/>
-        <color rgb="FFFF0000"/>
-        <rFont val="Calibri"/>
-        <family val="3"/>
-        <charset val="129"/>
-        <scheme val="minor"/>
-      </rPr>
-      <t>*</t>
-    </r>
-  </si>
-  <si>
     <t>Số tín chỉ còn nợ kỳ trước</t>
+  </si>
+  <si>
+    <t>Trạng thái trả nợ tín chỉ</t>
+  </si>
+  <si>
+    <t>Chuyên nghành</t>
   </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
-<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
+<styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <fonts count="9">
     <font>
       <sz val="11"/>
@@ -233,48 +221,51 @@
       <alignment vertical="center"/>
     </xf>
   </cellStyleXfs>
-  <cellXfs count="14">
+  <cellXfs count="15">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
     <xf numFmtId="0" fontId="3" fillId="2" borderId="1" xfId="0" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1">
-      <alignment vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1">
-      <alignment vertical="center"/>
-    </xf>
     <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
       <alignment vertical="center" wrapText="1"/>
     </xf>
     <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="3" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="49" fontId="6" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
-    </xf>
-    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="7" fillId="0" borderId="1" xfId="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" quotePrefix="1" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyBorder="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
+      <alignment vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="2" fillId="0" borderId="0" xfId="0" applyFont="1" applyAlignment="1">
       <alignment vertical="center"/>
     </xf>
-    <xf numFmtId="49" fontId="8" fillId="2" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
-      <alignment horizontal="center" vertical="center"/>
+    <xf numFmtId="49" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyAlignment="1">
+      <alignment vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment vertical="center"/>
     </xf>
   </cellXfs>
   <cellStyles count="2">
@@ -303,23 +294,23 @@
 <xdr:wsDr xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
   <xdr:twoCellAnchor>
     <xdr:from>
-      <xdr:col>5</xdr:col>
-      <xdr:colOff>1200150</xdr:colOff>
+      <xdr:col>4</xdr:col>
+      <xdr:colOff>1209675</xdr:colOff>
       <xdr:row>0</xdr:row>
-      <xdr:rowOff>19050</xdr:rowOff>
+      <xdr:rowOff>28575</xdr:rowOff>
     </xdr:from>
     <xdr:to>
-      <xdr:col>9</xdr:col>
+      <xdr:col>10</xdr:col>
       <xdr:colOff>1504950</xdr:colOff>
       <xdr:row>3</xdr:row>
-      <xdr:rowOff>104775</xdr:rowOff>
+      <xdr:rowOff>114300</xdr:rowOff>
     </xdr:to>
     <xdr:sp macro="" textlink="">
       <xdr:nvSpPr>
-        <xdr:cNvPr id="2" name="Rectangle 1">
+        <xdr:cNvPr id="3" name="Rectangle 2">
           <a:extLst>
             <a:ext uri="{FF2B5EF4-FFF2-40B4-BE49-F238E27FC236}">
-              <a16:creationId xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{99B488A7-E3E6-3D78-A753-2813B26BE3A8}"/>
+              <a16:creationId xmlns="" xmlns:a16="http://schemas.microsoft.com/office/drawing/2014/main" id="{99B488A7-E3E6-3D78-A753-2813B26BE3A8}"/>
             </a:ext>
           </a:extLst>
         </xdr:cNvPr>
@@ -327,8 +318,8 @@
       </xdr:nvSpPr>
       <xdr:spPr>
         <a:xfrm>
-          <a:off x="5610225" y="19050"/>
-          <a:ext cx="4238625" cy="561975"/>
+          <a:off x="3905250" y="28575"/>
+          <a:ext cx="8048625" cy="800100"/>
         </a:xfrm>
         <a:prstGeom prst="rect">
           <a:avLst/>
@@ -419,6 +410,17 @@
               </a:solidFill>
             </a:rPr>
             <a:t>- Giá trị cột số tín chỉ nợ ghi bằng số (VD: số tín chỉ nợ kỳ trước là hai-&gt; điền vào cột giá trị là 2)</a:t>
+          </a:r>
+        </a:p>
+        <a:p>
+          <a:pPr algn="l"/>
+          <a:r>
+            <a:rPr lang="en-US" sz="1100" kern="1200" baseline="0">
+              <a:solidFill>
+                <a:schemeClr val="tx1"/>
+              </a:solidFill>
+            </a:rPr>
+            <a:t>-Trạng thái trả nợ tín chỉ điền:Y(trả nợ xong), N(chưa trả xong)</a:t>
           </a:r>
           <a:endParaRPr lang="en-US" sz="1100" kern="1200">
             <a:solidFill>
@@ -729,173 +731,193 @@
 </file>
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
-<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{721892DF-7623-47C4-B30C-014733213156}">
-  <dimension ref="B1:J15"/>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
+  <dimension ref="B1:K15"/>
   <sheetFormatPr defaultColWidth="8.7109375" defaultRowHeight="15"/>
   <cols>
     <col min="1" max="1" width="2.42578125" customWidth="1"/>
-    <col min="2" max="2" width="4.7109375" customWidth="1"/>
-    <col min="3" max="3" width="18.7109375" style="7" customWidth="1"/>
-    <col min="4" max="4" width="16.7109375" style="7" bestFit="1" customWidth="1"/>
-    <col min="5" max="5" width="19.5703125" bestFit="1" customWidth="1"/>
-    <col min="6" max="6" width="18.140625" style="7" customWidth="1"/>
-    <col min="7" max="8" width="20.42578125" style="7" customWidth="1"/>
-    <col min="9" max="9" width="28.5703125" style="7" customWidth="1"/>
-    <col min="10" max="10" width="23.140625" style="7" customWidth="1"/>
+    <col min="2" max="2" width="4.7109375" style="4" customWidth="1"/>
+    <col min="3" max="3" width="18.7109375" style="2" customWidth="1"/>
+    <col min="4" max="4" width="14.5703125" style="2" customWidth="1"/>
+    <col min="5" max="5" width="24.140625" style="4" customWidth="1"/>
+    <col min="6" max="6" width="14.7109375" style="2" customWidth="1"/>
+    <col min="7" max="7" width="27.42578125" style="2" customWidth="1"/>
+    <col min="8" max="8" width="20.42578125" style="2" customWidth="1"/>
+    <col min="9" max="9" width="15.85546875" style="2" customWidth="1"/>
+    <col min="10" max="10" width="13.7109375" style="2" customWidth="1"/>
+    <col min="11" max="11" width="23.140625" style="2" customWidth="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="2:10" ht="18.75">
-      <c r="B1" s="1" t="s">
+    <row r="1" spans="2:11" s="14" customFormat="1" ht="18.75">
+      <c r="B1" s="12" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="2" spans="2:10" ht="18.75">
-      <c r="B2" s="1"/>
-    </row>
-    <row r="3" spans="2:10" ht="18.75">
-      <c r="B3" s="1"/>
-    </row>
-    <row r="4" spans="2:10">
-      <c r="C4" s="8"/>
-    </row>
-    <row r="5" spans="2:10" ht="17.25" customHeight="1">
-      <c r="B5" s="3" t="s">
+      <c r="C1" s="13"/>
+      <c r="D1" s="13"/>
+      <c r="F1" s="13"/>
+      <c r="G1" s="13"/>
+      <c r="H1" s="13"/>
+      <c r="I1" s="13"/>
+      <c r="J1" s="13"/>
+      <c r="K1" s="13"/>
+    </row>
+    <row r="2" spans="2:11" ht="18.75">
+      <c r="B2" s="11"/>
+    </row>
+    <row r="3" spans="2:11" ht="18.75">
+      <c r="B3" s="11"/>
+    </row>
+    <row r="5" spans="2:11" ht="36.75" customHeight="1">
+      <c r="B5" s="1" t="s">
         <v>0</v>
       </c>
-      <c r="C5" s="9" t="s">
+      <c r="C5" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="D5" s="10" t="s">
+      <c r="D5" s="3" t="s">
         <v>3</v>
       </c>
-      <c r="E5" s="11" t="s">
+      <c r="E5" s="5" t="s">
         <v>4</v>
       </c>
-      <c r="F5" s="13" t="s">
+      <c r="F5" s="6" t="s">
         <v>7</v>
       </c>
-      <c r="G5" s="4" t="s">
+      <c r="G5" s="1" t="s">
         <v>2</v>
       </c>
-      <c r="H5" s="4" t="s">
+      <c r="H5" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="I5" s="1" t="s">
         <v>8</v>
       </c>
-      <c r="I5" s="4" t="s">
+      <c r="J5" s="1" t="s">
         <v>9</v>
       </c>
-      <c r="J5" s="10" t="s">
+      <c r="K5" s="3" t="s">
         <v>5</v>
       </c>
     </row>
-    <row r="6" spans="2:10">
-      <c r="B6" s="2"/>
-      <c r="C6" s="12"/>
-      <c r="D6" s="5"/>
-      <c r="E6" s="5"/>
-      <c r="F6" s="5"/>
-      <c r="G6" s="5"/>
-      <c r="H6" s="5"/>
-      <c r="I6" s="5"/>
-      <c r="J6" s="6"/>
-    </row>
-    <row r="7" spans="2:10">
-      <c r="B7" s="2"/>
-      <c r="C7" s="12"/>
-      <c r="D7" s="6"/>
-      <c r="E7" s="6"/>
-      <c r="F7" s="6"/>
-      <c r="G7" s="6"/>
-      <c r="H7" s="6"/>
-      <c r="I7" s="6"/>
-      <c r="J7" s="6"/>
-    </row>
-    <row r="8" spans="2:10">
-      <c r="B8" s="2"/>
-      <c r="C8" s="6"/>
-      <c r="D8" s="6"/>
-      <c r="E8" s="6"/>
-      <c r="F8" s="6"/>
-      <c r="G8" s="6"/>
-      <c r="H8" s="6"/>
-      <c r="I8" s="6"/>
-      <c r="J8" s="6"/>
-    </row>
-    <row r="9" spans="2:10">
-      <c r="B9" s="2"/>
-      <c r="C9" s="6"/>
-      <c r="D9" s="6"/>
-      <c r="E9" s="6"/>
-      <c r="F9" s="6"/>
-      <c r="G9" s="6"/>
-      <c r="H9" s="6"/>
-      <c r="I9" s="6"/>
-      <c r="J9" s="6"/>
-    </row>
-    <row r="10" spans="2:10">
-      <c r="B10" s="2"/>
-      <c r="C10" s="6"/>
-      <c r="D10" s="6"/>
-      <c r="E10" s="6"/>
-      <c r="F10" s="6"/>
-      <c r="G10" s="6"/>
-      <c r="H10" s="6"/>
-      <c r="I10" s="6"/>
-      <c r="J10" s="6"/>
-    </row>
-    <row r="11" spans="2:10">
-      <c r="B11" s="2"/>
-      <c r="C11" s="6"/>
-      <c r="D11" s="6"/>
-      <c r="E11" s="6"/>
-      <c r="F11" s="6"/>
-      <c r="G11" s="6"/>
-      <c r="H11" s="6"/>
-      <c r="I11" s="6"/>
-      <c r="J11" s="6"/>
-    </row>
-    <row r="12" spans="2:10">
-      <c r="B12" s="2"/>
-      <c r="C12" s="6"/>
-      <c r="D12" s="6"/>
-      <c r="E12" s="6"/>
-      <c r="F12" s="6"/>
-      <c r="G12" s="6"/>
-      <c r="H12" s="6"/>
-      <c r="I12" s="6"/>
-      <c r="J12" s="6"/>
-    </row>
-    <row r="13" spans="2:10">
-      <c r="B13" s="2"/>
-      <c r="C13" s="6"/>
-      <c r="D13" s="6"/>
-      <c r="E13" s="6"/>
-      <c r="F13" s="6"/>
-      <c r="G13" s="6"/>
-      <c r="H13" s="6"/>
-      <c r="I13" s="6"/>
-      <c r="J13" s="6"/>
-    </row>
-    <row r="14" spans="2:10">
-      <c r="B14" s="2"/>
-      <c r="C14" s="6"/>
-      <c r="D14" s="6"/>
-      <c r="E14" s="6"/>
-      <c r="F14" s="6"/>
-      <c r="G14" s="6"/>
-      <c r="H14" s="6"/>
-      <c r="I14" s="6"/>
-      <c r="J14" s="6"/>
-    </row>
-    <row r="15" spans="2:10">
-      <c r="B15" s="2"/>
-      <c r="C15" s="6"/>
-      <c r="D15" s="6"/>
-      <c r="E15" s="6"/>
-      <c r="F15" s="6"/>
-      <c r="G15" s="6"/>
-      <c r="H15" s="6"/>
-      <c r="I15" s="6"/>
-      <c r="J15" s="6"/>
+    <row r="6" spans="2:11">
+      <c r="B6" s="10"/>
+      <c r="C6" s="7"/>
+      <c r="D6" s="8"/>
+      <c r="E6" s="8"/>
+      <c r="F6" s="8"/>
+      <c r="G6" s="8"/>
+      <c r="H6" s="8"/>
+      <c r="I6" s="8"/>
+      <c r="J6" s="8"/>
+      <c r="K6" s="9"/>
+    </row>
+    <row r="7" spans="2:11">
+      <c r="B7" s="10"/>
+      <c r="C7" s="7"/>
+      <c r="D7" s="9"/>
+      <c r="E7" s="9"/>
+      <c r="F7" s="9"/>
+      <c r="G7" s="9"/>
+      <c r="H7" s="9"/>
+      <c r="I7" s="9"/>
+      <c r="J7" s="9"/>
+      <c r="K7" s="9"/>
+    </row>
+    <row r="8" spans="2:11">
+      <c r="B8" s="10"/>
+      <c r="C8" s="9"/>
+      <c r="D8" s="9"/>
+      <c r="E8" s="9"/>
+      <c r="F8" s="9"/>
+      <c r="G8" s="9"/>
+      <c r="H8" s="9"/>
+      <c r="I8" s="9"/>
+      <c r="J8" s="9"/>
+      <c r="K8" s="9"/>
+    </row>
+    <row r="9" spans="2:11">
+      <c r="B9" s="10"/>
+      <c r="C9" s="9"/>
+      <c r="D9" s="9"/>
+      <c r="E9" s="9"/>
+      <c r="F9" s="9"/>
+      <c r="G9" s="9"/>
+      <c r="H9" s="9"/>
+      <c r="I9" s="9"/>
+      <c r="J9" s="9"/>
+      <c r="K9" s="9"/>
+    </row>
+    <row r="10" spans="2:11">
+      <c r="B10" s="10"/>
+      <c r="C10" s="9"/>
+      <c r="D10" s="9"/>
+      <c r="E10" s="9"/>
+      <c r="F10" s="9"/>
+      <c r="G10" s="9"/>
+      <c r="H10" s="9"/>
+      <c r="I10" s="9"/>
+      <c r="J10" s="9"/>
+      <c r="K10" s="9"/>
+    </row>
+    <row r="11" spans="2:11">
+      <c r="B11" s="10"/>
+      <c r="C11" s="9"/>
+      <c r="D11" s="9"/>
+      <c r="E11" s="9"/>
+      <c r="F11" s="9"/>
+      <c r="G11" s="9"/>
+      <c r="H11" s="9"/>
+      <c r="I11" s="9"/>
+      <c r="J11" s="9"/>
+      <c r="K11" s="9"/>
+    </row>
+    <row r="12" spans="2:11">
+      <c r="B12" s="10"/>
+      <c r="C12" s="9"/>
+      <c r="D12" s="9"/>
+      <c r="E12" s="9"/>
+      <c r="F12" s="9"/>
+      <c r="G12" s="9"/>
+      <c r="H12" s="9"/>
+      <c r="I12" s="9"/>
+      <c r="J12" s="9"/>
+      <c r="K12" s="9"/>
+    </row>
+    <row r="13" spans="2:11">
+      <c r="B13" s="10"/>
+      <c r="C13" s="9"/>
+      <c r="D13" s="9"/>
+      <c r="E13" s="9"/>
+      <c r="F13" s="9"/>
+      <c r="G13" s="9"/>
+      <c r="H13" s="9"/>
+      <c r="I13" s="9"/>
+      <c r="J13" s="9"/>
+      <c r="K13" s="9"/>
+    </row>
+    <row r="14" spans="2:11">
+      <c r="B14" s="10"/>
+      <c r="C14" s="9"/>
+      <c r="D14" s="9"/>
+      <c r="E14" s="9"/>
+      <c r="F14" s="9"/>
+      <c r="G14" s="9"/>
+      <c r="H14" s="9"/>
+      <c r="I14" s="9"/>
+      <c r="J14" s="9"/>
+      <c r="K14" s="9"/>
+    </row>
+    <row r="15" spans="2:11">
+      <c r="B15" s="10"/>
+      <c r="C15" s="9"/>
+      <c r="D15" s="9"/>
+      <c r="E15" s="9"/>
+      <c r="F15" s="9"/>
+      <c r="G15" s="9"/>
+      <c r="H15" s="9"/>
+      <c r="I15" s="9"/>
+      <c r="J15" s="9"/>
+      <c r="K15" s="9"/>
     </row>
   </sheetData>
   <phoneticPr fontId="1" type="noConversion"/>

</xml_diff>